<commit_message>
Update AsPersonProfile.fsh telecom emailType to 0..0 16fcfd8e4918ba4c7a578f972090d906437279d9
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dr-person.xlsx
+++ b/main/ig/StructureDefinition-as-dr-person.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-06T14:56:25+00:00</t>
+    <t>2025-03-12T15:24:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -6093,7 +6093,7 @@
         <v>78</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>77</v>

</xml_diff>